<commit_message>
updated bcs, crtpal, raf, shelf
</commit_message>
<xml_diff>
--- a/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
+++ b/InputData/ccs/BCS/BAU CCS Subsidy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\ccs\BCS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\Kentucky\KY-eps\InputData\ccs\BCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97EB2AB3-FE1A-4C06-98D6-C7F0874829B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91D34A5E-3AA7-46A0-86CA-BF4452182E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29670" yWindow="2655" windowWidth="26940" windowHeight="17250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -172,6 +172,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -700,43 +701,43 @@
       <c r="C2" s="4">
         <v>0</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="K2" s="7">
+      <c r="K2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="L2" s="7">
+      <c r="L2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>
-      <c r="M2" s="7">
+      <c r="M2" s="8">
         <f>'Electricity Calculations'!$B$4*About!$A$9</f>
         <v>40.035000000000004</v>
       </c>

</xml_diff>